<commit_message>
Correções gerais e adição de novos gráficos de tempo e comparativo
</commit_message>
<xml_diff>
--- a/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
+++ b/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
@@ -447,112 +447,112 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.89808175</v>
+        <v>0.89301155</v>
       </c>
       <c r="B2" t="n">
-        <v>13.25</v>
+        <v>16.59</v>
       </c>
       <c r="C2" t="n">
-        <v>16.26</v>
+        <v>20.99</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.88747263</v>
+        <v>0.88873252</v>
       </c>
       <c r="B3" t="n">
-        <v>14.97</v>
+        <v>14.53</v>
       </c>
       <c r="C3" t="n">
-        <v>5.51</v>
+        <v>20.58</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.88579645</v>
+        <v>0.87479243</v>
       </c>
       <c r="B4" t="n">
-        <v>14.61</v>
+        <v>17.62</v>
       </c>
       <c r="C4" t="n">
-        <v>12.36</v>
+        <v>20.51</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.8847155</v>
+        <v>0.84933421</v>
       </c>
       <c r="B5" t="n">
-        <v>6.13</v>
+        <v>12.19</v>
       </c>
       <c r="C5" t="n">
-        <v>10.76</v>
+        <v>23.57</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.88299962</v>
+        <v>0.8377738300000001</v>
       </c>
       <c r="B6" t="n">
-        <v>4.44</v>
+        <v>9.18</v>
       </c>
       <c r="C6" t="n">
-        <v>19.42</v>
+        <v>13.42</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.86906238</v>
+        <v>0.8303242199999999</v>
       </c>
       <c r="B7" t="n">
-        <v>7.46</v>
+        <v>15.69</v>
       </c>
       <c r="C7" t="n">
-        <v>13.16</v>
+        <v>16.45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.86288848</v>
+        <v>0.80788001</v>
       </c>
       <c r="B8" t="n">
-        <v>12.9</v>
+        <v>10.61</v>
       </c>
       <c r="C8" t="n">
-        <v>17.94</v>
+        <v>23.33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.86232149</v>
+        <v>0.80690974</v>
       </c>
       <c r="B9" t="n">
-        <v>17.19</v>
+        <v>16.89</v>
       </c>
       <c r="C9" t="n">
-        <v>10.8</v>
+        <v>12.23</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.8508697</v>
+        <v>0.80499069</v>
       </c>
       <c r="B10" t="n">
-        <v>17.82</v>
+        <v>17.62</v>
       </c>
       <c r="C10" t="n">
-        <v>6.92</v>
+        <v>13.1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.81077236</v>
+        <v>0.80494001</v>
       </c>
       <c r="B11" t="n">
-        <v>4.81</v>
+        <v>16.36</v>
       </c>
       <c r="C11" t="n">
-        <v>19.4</v>
+        <v>12.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correções gerais Adição de lógica de múltiplas populações Criação de classe de geração de gráficos Reorganização de pastas
</commit_message>
<xml_diff>
--- a/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
+++ b/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
@@ -447,112 +447,112 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.89301155</v>
+        <v>0.88784295</v>
       </c>
       <c r="B2" t="n">
-        <v>16.59</v>
+        <v>15.67</v>
       </c>
       <c r="C2" t="n">
-        <v>20.99</v>
+        <v>16.79</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.88873252</v>
+        <v>0.88630425</v>
       </c>
       <c r="B3" t="n">
-        <v>14.53</v>
+        <v>9.33</v>
       </c>
       <c r="C3" t="n">
-        <v>20.58</v>
+        <v>20.89</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.87479243</v>
+        <v>0.88453507</v>
       </c>
       <c r="B4" t="n">
-        <v>17.62</v>
+        <v>12.26</v>
       </c>
       <c r="C4" t="n">
-        <v>20.51</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.84933421</v>
+        <v>0.8789239</v>
       </c>
       <c r="B5" t="n">
-        <v>12.19</v>
+        <v>11.39</v>
       </c>
       <c r="C5" t="n">
-        <v>23.57</v>
+        <v>21.47</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.8377738300000001</v>
+        <v>0.8699893</v>
       </c>
       <c r="B6" t="n">
-        <v>9.18</v>
+        <v>17.7</v>
       </c>
       <c r="C6" t="n">
-        <v>13.42</v>
+        <v>16.52</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.8303242199999999</v>
+        <v>0.8602172</v>
       </c>
       <c r="B7" t="n">
-        <v>15.69</v>
+        <v>15.74</v>
       </c>
       <c r="C7" t="n">
-        <v>16.45</v>
+        <v>18.99</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.80788001</v>
+        <v>0.83121296</v>
       </c>
       <c r="B8" t="n">
-        <v>10.61</v>
+        <v>16.77</v>
       </c>
       <c r="C8" t="n">
-        <v>23.33</v>
+        <v>14.37</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.80690974</v>
+        <v>0.82637026</v>
       </c>
       <c r="B9" t="n">
-        <v>16.89</v>
+        <v>12.92</v>
       </c>
       <c r="C9" t="n">
-        <v>12.23</v>
+        <v>19.41</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.80499069</v>
+        <v>0.826183</v>
       </c>
       <c r="B10" t="n">
-        <v>17.62</v>
+        <v>16.15</v>
       </c>
       <c r="C10" t="n">
-        <v>13.1</v>
+        <v>19.55</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.80494001</v>
+        <v>0.8023514</v>
       </c>
       <c r="B11" t="n">
-        <v>16.36</v>
+        <v>10.85</v>
       </c>
       <c r="C11" t="n">
-        <v>12.21</v>
+        <v>18.64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Criação de lógica para estudo de parâmetros de forma combinatória. GA completo com 5 populacoes, graficos 4x6 e tabelas comparativas
</commit_message>
<xml_diff>
--- a/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
+++ b/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
@@ -447,112 +447,112 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.89656453</v>
+        <v>0.8885226000000001</v>
       </c>
       <c r="B2" t="n">
-        <v>16.8</v>
+        <v>13.7</v>
       </c>
       <c r="C2" t="n">
-        <v>13.32</v>
+        <v>12.87</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.88523057</v>
+        <v>0.8861565</v>
       </c>
       <c r="B3" t="n">
-        <v>15.51</v>
+        <v>10.77</v>
       </c>
       <c r="C3" t="n">
-        <v>23.92</v>
+        <v>16.47</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.88415034</v>
+        <v>0.88126047</v>
       </c>
       <c r="B4" t="n">
-        <v>18.07</v>
+        <v>15.64</v>
       </c>
       <c r="C4" t="n">
-        <v>18.22</v>
+        <v>22.71</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.88124833</v>
+        <v>0.87458691</v>
       </c>
       <c r="B5" t="n">
-        <v>9.99</v>
+        <v>12.38</v>
       </c>
       <c r="C5" t="n">
-        <v>13.22</v>
+        <v>14.82</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.86308859</v>
+        <v>0.87407362</v>
       </c>
       <c r="B6" t="n">
-        <v>15.19</v>
+        <v>16.41</v>
       </c>
       <c r="C6" t="n">
-        <v>12.68</v>
+        <v>20.87</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.86037298</v>
+        <v>0.85583833</v>
       </c>
       <c r="B7" t="n">
-        <v>10.87</v>
+        <v>11.43</v>
       </c>
       <c r="C7" t="n">
-        <v>16.22</v>
+        <v>13.71</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.83892677</v>
+        <v>0.85448778</v>
       </c>
       <c r="B8" t="n">
-        <v>13.01</v>
+        <v>12.96</v>
       </c>
       <c r="C8" t="n">
-        <v>17.82</v>
+        <v>13.17</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.83560169</v>
+        <v>0.85114279</v>
       </c>
       <c r="B9" t="n">
-        <v>13.58</v>
+        <v>16.12</v>
       </c>
       <c r="C9" t="n">
-        <v>19.31</v>
+        <v>12.78</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.82869009</v>
+        <v>0.84352344</v>
       </c>
       <c r="B10" t="n">
-        <v>13.53</v>
+        <v>9.34</v>
       </c>
       <c r="C10" t="n">
-        <v>18.6</v>
+        <v>14.05</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.82343278</v>
+        <v>0.8275273399999999</v>
       </c>
       <c r="B11" t="n">
-        <v>14.95</v>
+        <v>14.19</v>
       </c>
       <c r="C11" t="n">
-        <v>18.34</v>
+        <v>20.69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correção de leitura de componentes e individuos ja existentes
</commit_message>
<xml_diff>
--- a/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
+++ b/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
@@ -447,112 +447,112 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.8885226000000001</v>
+        <v>0.8948241</v>
       </c>
       <c r="B2" t="n">
-        <v>13.7</v>
+        <v>10.2</v>
       </c>
       <c r="C2" t="n">
-        <v>12.87</v>
+        <v>22.31</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.8861565</v>
+        <v>0.88840086</v>
       </c>
       <c r="B3" t="n">
-        <v>10.77</v>
+        <v>11.41</v>
       </c>
       <c r="C3" t="n">
-        <v>16.47</v>
+        <v>19.55</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.88126047</v>
+        <v>0.88702188</v>
       </c>
       <c r="B4" t="n">
-        <v>15.64</v>
+        <v>14.19</v>
       </c>
       <c r="C4" t="n">
-        <v>22.71</v>
+        <v>19.21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.87458691</v>
+        <v>0.87894002</v>
       </c>
       <c r="B5" t="n">
-        <v>12.38</v>
+        <v>9.43</v>
       </c>
       <c r="C5" t="n">
-        <v>14.82</v>
+        <v>12.64</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.87407362</v>
+        <v>0.86463113</v>
       </c>
       <c r="B6" t="n">
-        <v>16.41</v>
+        <v>16.08</v>
       </c>
       <c r="C6" t="n">
-        <v>20.87</v>
+        <v>22.85</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.85583833</v>
+        <v>0.85739387</v>
       </c>
       <c r="B7" t="n">
-        <v>11.43</v>
+        <v>13.77</v>
       </c>
       <c r="C7" t="n">
-        <v>13.71</v>
+        <v>15.22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.85448778</v>
+        <v>0.83210266</v>
       </c>
       <c r="B8" t="n">
-        <v>12.96</v>
+        <v>13.83</v>
       </c>
       <c r="C8" t="n">
-        <v>13.17</v>
+        <v>16.95</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.85114279</v>
+        <v>0.82784468</v>
       </c>
       <c r="B9" t="n">
-        <v>16.12</v>
+        <v>16.66</v>
       </c>
       <c r="C9" t="n">
-        <v>12.78</v>
+        <v>12.19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.84352344</v>
+        <v>0.82581889</v>
       </c>
       <c r="B10" t="n">
-        <v>9.34</v>
+        <v>16.08</v>
       </c>
       <c r="C10" t="n">
-        <v>14.05</v>
+        <v>14.54</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.8275273399999999</v>
+        <v>0.80596278</v>
       </c>
       <c r="B11" t="n">
-        <v>14.19</v>
+        <v>12.07</v>
       </c>
       <c r="C11" t="n">
-        <v>20.69</v>
+        <v>16.08</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Estudo de parametros completa
</commit_message>
<xml_diff>
--- a/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
+++ b/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
@@ -447,112 +447,112 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.89711118</v>
+        <v>0.89154669</v>
       </c>
       <c r="B2" t="n">
-        <v>9.19</v>
+        <v>16.31</v>
       </c>
       <c r="C2" t="n">
-        <v>21.1</v>
+        <v>23.29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.87482583</v>
+        <v>0.89032071</v>
       </c>
       <c r="B3" t="n">
-        <v>11.51</v>
+        <v>9.34</v>
       </c>
       <c r="C3" t="n">
-        <v>17.39</v>
+        <v>15.62</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.8525911900000001</v>
+        <v>0.86695202</v>
       </c>
       <c r="B4" t="n">
-        <v>17.79</v>
+        <v>15.38</v>
       </c>
       <c r="C4" t="n">
-        <v>14.29</v>
+        <v>14.44</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.84925904</v>
+        <v>0.85719069</v>
       </c>
       <c r="B5" t="n">
-        <v>17.01</v>
+        <v>17.62</v>
       </c>
       <c r="C5" t="n">
-        <v>22.81</v>
+        <v>15.23</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.84761177</v>
+        <v>0.85252222</v>
       </c>
       <c r="B6" t="n">
-        <v>10.54</v>
+        <v>15.93</v>
       </c>
       <c r="C6" t="n">
-        <v>21.29</v>
+        <v>12.71</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.83685822</v>
+        <v>0.82246193</v>
       </c>
       <c r="B7" t="n">
-        <v>12.71</v>
+        <v>15.13</v>
       </c>
       <c r="C7" t="n">
-        <v>13.36</v>
+        <v>22.93</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.83610448</v>
+        <v>0.82198298</v>
       </c>
       <c r="B8" t="n">
-        <v>14.38</v>
+        <v>11.96</v>
       </c>
       <c r="C8" t="n">
-        <v>14.15</v>
+        <v>18.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.8335991699999999</v>
+        <v>0.80939348</v>
       </c>
       <c r="B9" t="n">
-        <v>17.86</v>
+        <v>9.34</v>
       </c>
       <c r="C9" t="n">
-        <v>16.08</v>
+        <v>20.82</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.81232423</v>
+        <v>0.80882923</v>
       </c>
       <c r="B10" t="n">
-        <v>11.16</v>
+        <v>12.86</v>
       </c>
       <c r="C10" t="n">
-        <v>12.27</v>
+        <v>18.35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.80533681</v>
+        <v>0.80617999</v>
       </c>
       <c r="B11" t="n">
-        <v>14.96</v>
+        <v>15.19</v>
       </c>
       <c r="C11" t="n">
-        <v>17.12</v>
+        <v>20.15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correções e novos gráficos
</commit_message>
<xml_diff>
--- a/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
+++ b/Cenário em Ponte/Cromossomo NT/Geradores/Excel/componentes.xlsx
@@ -447,112 +447,112 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.89154669</v>
+        <v>0.87464334</v>
       </c>
       <c r="B2" t="n">
-        <v>16.31</v>
+        <v>16.18</v>
       </c>
       <c r="C2" t="n">
-        <v>23.29</v>
+        <v>22.84</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>0.89032071</v>
+        <v>0.87227966</v>
       </c>
       <c r="B3" t="n">
-        <v>9.34</v>
+        <v>15.46</v>
       </c>
       <c r="C3" t="n">
-        <v>15.62</v>
+        <v>15.26</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0.86695202</v>
+        <v>0.86040638</v>
       </c>
       <c r="B4" t="n">
-        <v>15.38</v>
+        <v>16.94</v>
       </c>
       <c r="C4" t="n">
-        <v>14.44</v>
+        <v>20.13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.85719069</v>
+        <v>0.85577812</v>
       </c>
       <c r="B5" t="n">
-        <v>17.62</v>
+        <v>11.51</v>
       </c>
       <c r="C5" t="n">
-        <v>15.23</v>
+        <v>15.63</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.85252222</v>
+        <v>0.853419</v>
       </c>
       <c r="B6" t="n">
-        <v>15.93</v>
+        <v>13.07</v>
       </c>
       <c r="C6" t="n">
-        <v>12.71</v>
+        <v>17.46</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.82246193</v>
+        <v>0.84137089</v>
       </c>
       <c r="B7" t="n">
-        <v>15.13</v>
+        <v>14.5</v>
       </c>
       <c r="C7" t="n">
-        <v>22.93</v>
+        <v>12.27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.82198298</v>
+        <v>0.84129642</v>
       </c>
       <c r="B8" t="n">
-        <v>11.96</v>
+        <v>13.59</v>
       </c>
       <c r="C8" t="n">
-        <v>18.4</v>
+        <v>16.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.80939348</v>
+        <v>0.83459235</v>
       </c>
       <c r="B9" t="n">
-        <v>9.34</v>
+        <v>11.49</v>
       </c>
       <c r="C9" t="n">
-        <v>20.82</v>
+        <v>12.38</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.80882923</v>
+        <v>0.82382803</v>
       </c>
       <c r="B10" t="n">
-        <v>12.86</v>
+        <v>14.07</v>
       </c>
       <c r="C10" t="n">
-        <v>18.35</v>
+        <v>20.87</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.80617999</v>
+        <v>0.81494565</v>
       </c>
       <c r="B11" t="n">
-        <v>15.19</v>
+        <v>15.45</v>
       </c>
       <c r="C11" t="n">
-        <v>20.15</v>
+        <v>19.16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>